<commit_message>
chore: 가계부_2026_v0.05.xlsx 재생성 (ColorScaleRule 색상 보정 반영)
https://claude.ai/code/session_016ow6E7GTWFCMp2FCZEfAVy
</commit_message>
<xml_diff>
--- a/money-log/data/가계부_2026_v0.05.xlsx
+++ b/money-log/data/가계부_2026_v0.05.xlsx
@@ -58,7 +58,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001A2B4A"/>
+      <color rgb="001E293B"/>
       <sz val="12"/>
     </font>
     <font>
@@ -70,7 +70,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00C0392B"/>
+      <color rgb="00DC2626"/>
       <sz val="12"/>
     </font>
     <font>
@@ -103,12 +103,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00C0392B"/>
+      <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri Light"/>
-      <color rgb="001A2B4A"/>
+      <color rgb="001E293B"/>
       <sz val="16"/>
     </font>
     <font>
@@ -118,7 +118,7 @@
     </font>
     <font>
       <name val="Calibri Light"/>
-      <color rgb="001A2B4A"/>
+      <color rgb="001E293B"/>
       <sz val="18"/>
     </font>
     <font>
@@ -134,18 +134,18 @@
     </font>
     <font>
       <name val="Calibri Light"/>
-      <color rgb="001A2B4A"/>
+      <color rgb="001E293B"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="001A2B4A"/>
+      <color rgb="001E293B"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001A2B4A"/>
+      <color rgb="001E293B"/>
       <sz val="11"/>
     </font>
     <font>
@@ -164,17 +164,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6EAF8"/>
+        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002471A3"/>
+        <fgColor rgb="002563EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A2B4A"/>
+        <fgColor rgb="001E293B"/>
       </patternFill>
     </fill>
     <fill>
@@ -189,32 +189,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E8449"/>
+        <fgColor rgb="0016A34A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F8F0"/>
+        <fgColor rgb="00F0FDF4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C0392B"/>
+        <fgColor rgb="00DC2626"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDF2F2"/>
+        <fgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004A5568"/>
+        <fgColor rgb="00475569"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFB"/>
+        <fgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -661,8 +661,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFD0D0"/>
-          <bgColor rgb="00FFD0D0"/>
+          <fgColor rgb="00FEE2E2"/>
+          <bgColor rgb="00FEE2E2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -794,7 +794,7 @@
           </tx>
           <spPr>
             <a:solidFill>
-              <a:srgbClr val="1E8449"/>
+              <a:srgbClr val="16A34A"/>
             </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
@@ -819,7 +819,7 @@
           </tx>
           <spPr>
             <a:solidFill>
-              <a:srgbClr val="C0392B"/>
+              <a:srgbClr val="DC2626"/>
             </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
@@ -851,7 +851,7 @@
           <spPr>
             <a:ln w="20000">
               <a:solidFill>
-                <a:srgbClr val="1E8449"/>
+                <a:srgbClr val="16A34A"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -885,7 +885,7 @@
           <spPr>
             <a:ln w="20000">
               <a:solidFill>
-                <a:srgbClr val="C0392B"/>
+                <a:srgbClr val="DC2626"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1005,7 +1005,7 @@
           <spPr>
             <a:ln w="28000">
               <a:solidFill>
-                <a:srgbClr val="2471A3"/>
+                <a:srgbClr val="2563EB"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1125,7 +1125,7 @@
           </tx>
           <spPr>
             <a:solidFill>
-              <a:srgbClr val="2471A3"/>
+              <a:srgbClr val="2563EB"/>
             </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
@@ -1150,7 +1150,7 @@
           </tx>
           <spPr>
             <a:solidFill>
-              <a:srgbClr val="C0392B"/>
+              <a:srgbClr val="DC2626"/>
             </a:solidFill>
             <a:ln>
               <a:prstDash val="solid"/>
@@ -15755,7 +15755,7 @@
         <cfvo type="percentile" val="100"/>
         <color rgb="FFFFFFFF"/>
         <color rgb="FFFFEB84"/>
-        <color rgb="FFC0392B"/>
+        <color rgb="FFDC2626"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -41040,7 +41040,7 @@
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
-        <color rgb="002471A3"/>
+        <color rgb="002563EB"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>

</xml_diff>